<commit_message>
Advance trade elasticities econometric workflow
</commit_message>
<xml_diff>
--- a/trade-elasticities-cointegration/outputs/section_10_cointegration_results.xlsx
+++ b/trade-elasticities-cointegration/outputs/section_10_cointegration_results.xlsx
@@ -7,12 +7,13 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="equations" sheetId="1" r:id="rId1"/>
-    <sheet name="long_run_coefficients" sheetId="2" r:id="rId2"/>
-    <sheet name="engle_granger" sheetId="3" r:id="rId3"/>
-    <sheet name="gregory_hansen" sheetId="4" r:id="rId4"/>
-    <sheet name="decision_summary" sheetId="5" r:id="rId5"/>
-    <sheet name="residuals" sheetId="6" r:id="rId6"/>
+    <sheet name="model_sample" sheetId="1" r:id="rId1"/>
+    <sheet name="equations" sheetId="2" r:id="rId2"/>
+    <sheet name="long_run_coefficients" sheetId="3" r:id="rId3"/>
+    <sheet name="engle_granger" sheetId="4" r:id="rId4"/>
+    <sheet name="gregory_hansen" sheetId="5" r:id="rId5"/>
+    <sheet name="decision_summary" sheetId="6" r:id="rId6"/>
+    <sheet name="residuals" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -360,151 +361,41 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="20.7109375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>model_key</t>
+          <t>model_sample_start</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>model_label</t>
+          <t>model_sample_end</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>method</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>dependent_var</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>regressors</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>n_obs</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>first_quarter</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>last_quarter</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>r_squared</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>adj_r_squared</t>
+          <t>model_sample_note</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>imports</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Importaciones: comercio, PIB argentino e ITCRM</t>
-        </is>
+      <c r="A2" s="2">
+        <v>37987</v>
+      </c>
+      <c r="B2" s="2">
+        <v>44835</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Engle-Granger first-stage OLS</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>ln_imports_real</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>ln_gdp_real + ln_itcrm</t>
-        </is>
-      </c>
-      <c r="F2">
-        <v>76</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2004Q1</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2022Q4</t>
-        </is>
-      </c>
-      <c r="I2">
-        <v>0.8609397778547253</v>
-      </c>
-      <c r="J2">
-        <v>0.8571299087548547</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>exports</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Exportaciones: comercio, PIB socios e ITCRM</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Engle-Granger first-stage OLS</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>ln_exports_real</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>ln_pib_socios + ln_itcrm</t>
-        </is>
-      </c>
-      <c r="F3">
-        <v>76</v>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2004Q1</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2022Q4</t>
-        </is>
-      </c>
-      <c r="I3">
-        <v>0.2099367593767753</v>
-      </c>
-      <c r="J3">
-        <v>0.1882911911405224</v>
+          <t>Muestra econometrica comun para estacionariedad, cointegracion y modelos; las visualizaciones conservan la cobertura completa para documentar disponibilidad temporal.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -514,7 +405,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -530,27 +421,42 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>term</t>
+          <t>method</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>estimate</t>
+          <t>dependent_var</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>std_error</t>
+          <t>regressors</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>t_statistic</t>
+          <t>n_obs</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>p_value</t>
+          <t>first_quarter</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>last_quarter</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>r_squared</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>adj_r_squared</t>
         </is>
       </c>
     </row>
@@ -567,165 +473,83 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>(Intercept)</t>
-        </is>
-      </c>
-      <c r="D2">
-        <v>-6.494961641383456</v>
-      </c>
-      <c r="E2">
-        <v>2.340347392359403</v>
+          <t>Engle-Granger first-stage OLS</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ln_imports_real</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ln_gdp_real + ln_itcrm</t>
+        </is>
       </c>
       <c r="F2">
-        <v>-2.775212629794934</v>
-      </c>
-      <c r="G2">
-        <v>0.007002019218821045</v>
+        <v>76</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2004Q1</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2022Q4</t>
+        </is>
+      </c>
+      <c r="I2">
+        <v>0.8609397778547253</v>
+      </c>
+      <c r="J2">
+        <v>0.8571299087548547</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>imports</t>
+          <t>exports</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Importaciones: comercio, PIB argentino e ITCRM</t>
+          <t>Exportaciones: comercio, PIB socios e ITCRM</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ln_gdp_real</t>
-        </is>
-      </c>
-      <c r="D3">
-        <v>1.518408430994575</v>
-      </c>
-      <c r="E3">
-        <v>0.1507837929940569</v>
+          <t>Engle-Granger first-stage OLS</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ln_exports_real</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ln_pib_socios + ln_itcrm</t>
+        </is>
       </c>
       <c r="F3">
-        <v>10.07010369512606</v>
-      </c>
-      <c r="G3">
-        <v>1.890890497492488E-15</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>imports</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Importaciones: comercio, PIB argentino e ITCRM</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>ln_itcrm</t>
-        </is>
-      </c>
-      <c r="D4">
-        <v>-0.3991932036902151</v>
-      </c>
-      <c r="E4">
-        <v>0.08472768698826195</v>
-      </c>
-      <c r="F4">
-        <v>-4.711484732794827</v>
-      </c>
-      <c r="G4">
-        <v>1.145399526078436E-05</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>exports</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Exportaciones: comercio, PIB socios e ITCRM</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>(Intercept)</t>
-        </is>
-      </c>
-      <c r="D5">
-        <v>7.61789640486439</v>
-      </c>
-      <c r="E5">
-        <v>1.276686768322203</v>
-      </c>
-      <c r="F5">
-        <v>5.966926730881435</v>
-      </c>
-      <c r="G5">
-        <v>7.99231997032852E-08</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>exports</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Exportaciones: comercio, PIB socios e ITCRM</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>ln_pib_socios</t>
-        </is>
-      </c>
-      <c r="D6">
-        <v>0.7203209712546355</v>
-      </c>
-      <c r="E6">
-        <v>0.1879806797509279</v>
-      </c>
-      <c r="F6">
-        <v>3.831888320698977</v>
-      </c>
-      <c r="G6">
-        <v>0.0002669689191450794</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>exports</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Exportaciones: comercio, PIB socios e ITCRM</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>ln_itcrm</t>
-        </is>
-      </c>
-      <c r="D7">
-        <v>0.1593885399165426</v>
-      </c>
-      <c r="E7">
-        <v>0.08828862715085903</v>
-      </c>
-      <c r="F7">
-        <v>1.805312247569496</v>
-      </c>
-      <c r="G7">
-        <v>0.07514911099825242</v>
+        <v>76</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2004Q1</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2022Q4</t>
+        </is>
+      </c>
+      <c r="I3">
+        <v>0.2099367593767753</v>
+      </c>
+      <c r="J3">
+        <v>0.1882911911405224</v>
       </c>
     </row>
   </sheetData>
@@ -735,7 +559,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -751,47 +575,27 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>method</t>
+          <t>term</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>dependent_var</t>
+          <t>estimate</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>regressors</t>
+          <t>std_error</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>n_obs</t>
+          <t>t_statistic</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>adf_lag</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>statistic</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
           <t>p_value</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>conclusion_5pct</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>note</t>
         </is>
       </c>
     </row>
@@ -808,89 +612,165 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Engle-Granger residual ADF</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>ln_imports_real</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>ln_gdp_real + ln_itcrm</t>
-        </is>
+          <t>(Intercept)</t>
+        </is>
+      </c>
+      <c r="D2">
+        <v>-6.494961641383456</v>
+      </c>
+      <c r="E2">
+        <v>2.340347392359403</v>
       </c>
       <c r="F2">
-        <v>76</v>
+        <v>-2.775212629794934</v>
       </c>
       <c r="G2">
-        <v>4</v>
-      </c>
-      <c r="H2">
-        <v>-4.483205277778568</v>
-      </c>
-      <c r="I2">
-        <v>0.01</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>residuos estacionarios; cointegracion</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>ADF aplicado sobre residuos de la primera etapa; la decision debe interpretarse como evidencia preliminar.</t>
-        </is>
+        <v>0.007002019218821045</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>exports</t>
+          <t>imports</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>Importaciones: comercio, PIB argentino e ITCRM</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ln_gdp_real</t>
+        </is>
+      </c>
+      <c r="D3">
+        <v>1.518408430994575</v>
+      </c>
+      <c r="E3">
+        <v>0.1507837929940569</v>
+      </c>
+      <c r="F3">
+        <v>10.07010369512606</v>
+      </c>
+      <c r="G3">
+        <v>1.890890497492488E-15</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>imports</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Importaciones: comercio, PIB argentino e ITCRM</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ln_itcrm</t>
+        </is>
+      </c>
+      <c r="D4">
+        <v>-0.3991932036902151</v>
+      </c>
+      <c r="E4">
+        <v>0.08472768698826195</v>
+      </c>
+      <c r="F4">
+        <v>-4.711484732794827</v>
+      </c>
+      <c r="G4">
+        <v>1.145399526078436E-05</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>exports</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>Exportaciones: comercio, PIB socios e ITCRM</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Engle-Granger residual ADF</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>ln_exports_real</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>ln_pib_socios + ln_itcrm</t>
-        </is>
-      </c>
-      <c r="F3">
-        <v>76</v>
-      </c>
-      <c r="G3">
-        <v>4</v>
-      </c>
-      <c r="H3">
-        <v>-3.770587871669464</v>
-      </c>
-      <c r="I3">
-        <v>0.02474600583320619</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>residuos estacionarios; cointegracion</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>ADF aplicado sobre residuos de la primera etapa; la decision debe interpretarse como evidencia preliminar.</t>
-        </is>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>(Intercept)</t>
+        </is>
+      </c>
+      <c r="D5">
+        <v>7.61789640486439</v>
+      </c>
+      <c r="E5">
+        <v>1.276686768322203</v>
+      </c>
+      <c r="F5">
+        <v>5.966926730881435</v>
+      </c>
+      <c r="G5">
+        <v>7.99231997032852E-08</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>exports</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Exportaciones: comercio, PIB socios e ITCRM</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ln_pib_socios</t>
+        </is>
+      </c>
+      <c r="D6">
+        <v>0.7203209712546355</v>
+      </c>
+      <c r="E6">
+        <v>0.1879806797509279</v>
+      </c>
+      <c r="F6">
+        <v>3.831888320698977</v>
+      </c>
+      <c r="G6">
+        <v>0.0002669689191450794</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>exports</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Exportaciones: comercio, PIB socios e ITCRM</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ln_itcrm</t>
+        </is>
+      </c>
+      <c r="D7">
+        <v>0.1593885399165426</v>
+      </c>
+      <c r="E7">
+        <v>0.08828862715085903</v>
+      </c>
+      <c r="F7">
+        <v>1.805312247569496</v>
+      </c>
+      <c r="G7">
+        <v>0.07514911099825242</v>
       </c>
     </row>
   </sheetData>
@@ -900,7 +780,172 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:K3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>model_key</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>model_label</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>method</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>dependent_var</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>regressors</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>n_obs</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>adf_lag</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>statistic</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>p_value</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>conclusion_5pct</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>imports</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Importaciones: comercio, PIB argentino e ITCRM</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Engle-Granger residual ADF</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ln_imports_real</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ln_gdp_real + ln_itcrm</t>
+        </is>
+      </c>
+      <c r="F2">
+        <v>76</v>
+      </c>
+      <c r="G2">
+        <v>4</v>
+      </c>
+      <c r="H2">
+        <v>-4.483205277778568</v>
+      </c>
+      <c r="I2">
+        <v>0.01</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>residuos estacionarios; cointegracion</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>ADF aplicado sobre residuos de la primera etapa; el p-value del ADF estandar se reporta como aproximacion; la inferencia formal de Engle-Granger requiere valores criticos especificos para residuos de cointegracion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>exports</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Exportaciones: comercio, PIB socios e ITCRM</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Engle-Granger residual ADF</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ln_exports_real</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ln_pib_socios + ln_itcrm</t>
+        </is>
+      </c>
+      <c r="F3">
+        <v>76</v>
+      </c>
+      <c r="G3">
+        <v>4</v>
+      </c>
+      <c r="H3">
+        <v>-3.770587871669464</v>
+      </c>
+      <c r="I3">
+        <v>0.02474600583320619</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>residuos estacionarios; cointegracion</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ADF aplicado sobre residuos de la primera etapa; el p-value del ADF estandar se reporta como aproximacion; la inferencia formal de Engle-Granger requiere valores criticos especificos para residuos de cointegracion.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:N7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="6" max="6" width="20.7109375" style="2" customWidth="1"/>
@@ -959,10 +1004,20 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>critical_value_source</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>trimming</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>conclusion_5pct</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -1009,12 +1064,20 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
+          <t>aproximado; verificar contra tabla del curso o bibliografia antes de reportar como resultado definitivo</t>
+        </is>
+      </c>
+      <c r="L2">
+        <v>0.15</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
           <t>rechaza no cointegracion con quiebre</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Valores criticos aproximados para Gregory-Hansen con dos regresores; confirmar contra tabla del curso si se reporta como resultado final.</t>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Valores criticos aproximados para Gregory-Hansen con dos regresores; no presentar como resultado definitivo sin validar los valores criticos contra el material del curso o la bibliografia.</t>
         </is>
       </c>
     </row>
@@ -1059,12 +1122,20 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
+          <t>aproximado; verificar contra tabla del curso o bibliografia antes de reportar como resultado definitivo</t>
+        </is>
+      </c>
+      <c r="L3">
+        <v>0.15</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
           <t>no rechaza no cointegracion con quiebre</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Valores criticos aproximados para Gregory-Hansen con dos regresores; confirmar contra tabla del curso si se reporta como resultado final.</t>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Valores criticos aproximados para Gregory-Hansen con dos regresores; no presentar como resultado definitivo sin validar los valores criticos contra el material del curso o la bibliografia.</t>
         </is>
       </c>
     </row>
@@ -1109,12 +1180,20 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
+          <t>aproximado; verificar contra tabla del curso o bibliografia antes de reportar como resultado definitivo</t>
+        </is>
+      </c>
+      <c r="L4">
+        <v>0.15</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
           <t>no rechaza no cointegracion con quiebre</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Valores criticos aproximados para Gregory-Hansen con dos regresores; confirmar contra tabla del curso si se reporta como resultado final.</t>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Valores criticos aproximados para Gregory-Hansen con dos regresores; no presentar como resultado definitivo sin validar los valores criticos contra el material del curso o la bibliografia.</t>
         </is>
       </c>
     </row>
@@ -1159,12 +1238,20 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
+          <t>aproximado; verificar contra tabla del curso o bibliografia antes de reportar como resultado definitivo</t>
+        </is>
+      </c>
+      <c r="L5">
+        <v>0.15</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
           <t>no rechaza no cointegracion con quiebre</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Valores criticos aproximados para Gregory-Hansen con dos regresores; confirmar contra tabla del curso si se reporta como resultado final.</t>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Valores criticos aproximados para Gregory-Hansen con dos regresores; no presentar como resultado definitivo sin validar los valores criticos contra el material del curso o la bibliografia.</t>
         </is>
       </c>
     </row>
@@ -1209,12 +1296,20 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
+          <t>aproximado; verificar contra tabla del curso o bibliografia antes de reportar como resultado definitivo</t>
+        </is>
+      </c>
+      <c r="L6">
+        <v>0.15</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
           <t>no rechaza no cointegracion con quiebre</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>Valores criticos aproximados para Gregory-Hansen con dos regresores; confirmar contra tabla del curso si se reporta como resultado final.</t>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Valores criticos aproximados para Gregory-Hansen con dos regresores; no presentar como resultado definitivo sin validar los valores criticos contra el material del curso o la bibliografia.</t>
         </is>
       </c>
     </row>
@@ -1259,12 +1354,20 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
+          <t>aproximado; verificar contra tabla del curso o bibliografia antes de reportar como resultado definitivo</t>
+        </is>
+      </c>
+      <c r="L7">
+        <v>0.15</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
           <t>no rechaza no cointegracion con quiebre</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>Valores criticos aproximados para Gregory-Hansen con dos regresores; confirmar contra tabla del curso si se reporta como resultado final.</t>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Valores criticos aproximados para Gregory-Hansen con dos regresores; no presentar como resultado definitivo sin validar los valores criticos contra el material del curso o la bibliografia.</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1376,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1427,7 +1530,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E153"/>
   <sheetFormatPr defaultRowHeight="15"/>

</xml_diff>